<commit_message>
Atualiza dados do estoque e compras2
</commit_message>
<xml_diff>
--- a/data-source/COMPRAPARAGUAI.xlsx
+++ b/data-source/COMPRAPARAGUAI.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/Relatórios SMART-STOCK/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/SMART-STOCK/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{0945D746-136B-4EA6-8FA1-116932EBA3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA4EAF21-63DB-4AC9-8F09-C439AA7B8772}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{0945D746-136B-4EA6-8FA1-116932EBA3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1C1D375-55D7-4880-8691-307D65AA5FC1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EC661E31-7BDC-4492-BDCF-C8B212342257}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
   <si>
     <t>Produto</t>
   </si>
@@ -137,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -145,6 +145,7 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65630E9C-5564-429A-8139-A7EDF74685C9}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
@@ -557,6 +558,40 @@
         <v>30610</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>15721</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>21000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>9010</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>10000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>